<commit_message>
docs: alinha casos de uso ao fluxo e atualiza cronograma
</commit_message>
<xml_diff>
--- a/docs/planejamento/Cronograma_TCC_Gestao_Integrada.xlsx
+++ b/docs/planejamento/Cronograma_TCC_Gestao_Integrada.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cronograma" sheetId="1" r:id="R292296cb88e24e38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legenda" sheetId="2" r:id="R8d199b49031e4d6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gantt Semanal" sheetId="3" r:id="R9571ed773c5542fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cronograma" sheetId="1" r:id="R295fddf1f38e4229"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legenda" sheetId="2" r:id="R94cec3b7cde94ca7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gantt Semanal" sheetId="3" r:id="R5f3daae2dbf045c7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -47,7 +47,7 @@
       <x:color rgb="FFFFFFFF"/>
     </x:font>
   </x:fonts>
-  <x:fills count="15">
+  <x:fills count="16">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -119,6 +119,11 @@
         <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -132,7 +137,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="48">
+  <x:cellXfs count="49">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
@@ -247,11 +252,12 @@
     <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="6">
+  <x:dxfs count="21">
     <x:dxf>
       <x:fill>
         <x:patternFill>
@@ -275,22 +281,127 @@
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFC6E0B4"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE699"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF4CCCC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFF4CCCC"/>
+          <x:bgColor rgb="FFD9EAF7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFD9EAF7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFD9EAF7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFD9EAF7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFD9EAF7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFE2F0D9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFE2F0D9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFE2F0D9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFE2F0D9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -803,15 +914,15 @@
       <x:c r="B9" s="6" t="str">
         <x:v>Finalizar e validar o fluxograma macro com o grupo</x:v>
       </x:c>
-      <x:c r="C9" s="34" t="n">
-        <x:v>46308</x:v>
-      </x:c>
-      <x:c r="D9" s="34" t="n">
-        <x:v>46311</x:v>
+      <x:c r="C9" s="34" t="d">
+        <x:v>2026-10-20T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D9" s="34" t="d">
+        <x:v>2026-10-22T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="E9" s="6" t="n">
         <x:f>D9-C9+1</x:f>
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F9" s="6" t="str">
         <x:v>TCC1</x:v>
@@ -821,7 +932,7 @@
       </x:c>
       <x:c r="H9" s="6"/>
       <x:c r="I9" s="6" t="str">
-        <x:v>Todo pedido gera uma OP, mesmo com estoque acabado suficiente</x:v>
+        <x:v>Uma OP gerada automaticamente no registro de cada pedido</x:v>
       </x:c>
       <x:c r="J9" s="8" t="n">
         <x:v>0</x:v>
@@ -836,15 +947,15 @@
       <x:c r="B10" s="6" t="str">
         <x:v>Atualizar escopo, requisitos e regras de negócio</x:v>
       </x:c>
-      <x:c r="C10" s="34" t="n">
-        <x:v>46308</x:v>
-      </x:c>
-      <x:c r="D10" s="34" t="n">
-        <x:v>46313</x:v>
+      <x:c r="C10" s="34" t="d">
+        <x:v>2026-10-20T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D10" s="34" t="d">
+        <x:v>2026-10-24T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="E10" s="6" t="n">
         <x:f>D10-C10+1</x:f>
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="F10" s="6" t="inlineStr">
         <x:is>
@@ -877,11 +988,11 @@
       <x:c r="B11" s="6" t="str">
         <x:v>Finalizar atores, casos de uso e responsabilidades</x:v>
       </x:c>
-      <x:c r="C11" s="34" t="n">
-        <x:v>46314</x:v>
-      </x:c>
-      <x:c r="D11" s="34" t="n">
-        <x:v>46318</x:v>
+      <x:c r="C11" s="34" t="d">
+        <x:v>2026-10-21T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D11" s="34" t="d">
+        <x:v>2026-10-25T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="E11" s="6" t="n">
         <x:f>D11-C11+1</x:f>
@@ -918,15 +1029,15 @@
       <x:c r="B12" s="6" t="str">
         <x:v>Diagrama de casos de uso + descrições principais</x:v>
       </x:c>
-      <x:c r="C12" s="34" t="n">
-        <x:v>46314</x:v>
-      </x:c>
-      <x:c r="D12" s="34" t="n">
-        <x:v>46320</x:v>
+      <x:c r="C12" s="34" t="d">
+        <x:v>2026-10-23T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D12" s="34" t="d">
+        <x:v>2026-10-27T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="E12" s="6" t="n">
         <x:f>D12-C12+1</x:f>
-        <x:v>7</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="F12" s="6" t="inlineStr">
         <x:is>
@@ -957,15 +1068,15 @@
       <x:c r="B13" s="6" t="str">
         <x:v>Diagrama de classes de domínio</x:v>
       </x:c>
-      <x:c r="C13" s="34" t="n">
-        <x:v>46317</x:v>
-      </x:c>
-      <x:c r="D13" s="34" t="n">
-        <x:v>46323</x:v>
+      <x:c r="C13" s="34" t="d">
+        <x:v>2026-10-25T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D13" s="34" t="d">
+        <x:v>2026-10-30T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="E13" s="6" t="n">
         <x:f>D13-C13+1</x:f>
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="F13" s="6" t="inlineStr">
         <x:is>
@@ -994,11 +1105,11 @@
       <x:c r="B14" s="9" t="str">
         <x:v>DER e modelagem do banco de dados</x:v>
       </x:c>
-      <x:c r="C14" s="37" t="n">
-        <x:v>46321</x:v>
-      </x:c>
-      <x:c r="D14" s="37" t="n">
-        <x:v>46326</x:v>
+      <x:c r="C14" s="37" t="d">
+        <x:v>2026-10-28T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D14" s="37" t="d">
+        <x:v>2026-11-02T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="E14" s="9" t="n">
         <x:f>D14-C14+1</x:f>
@@ -1035,15 +1146,15 @@
       <x:c r="B15" s="9" t="str">
         <x:v>Diagramas de atividades dos fluxos principais</x:v>
       </x:c>
-      <x:c r="C15" s="37" t="n">
-        <x:v>46324</x:v>
-      </x:c>
-      <x:c r="D15" s="37" t="n">
-        <x:v>46330</x:v>
+      <x:c r="C15" s="37" t="d">
+        <x:v>2026-10-31T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D15" s="37" t="d">
+        <x:v>2026-11-05T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="E15" s="9" t="n">
         <x:f>D15-C15+1</x:f>
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="F15" s="9" t="inlineStr">
         <x:is>
@@ -1074,15 +1185,15 @@
       <x:c r="B16" s="9" t="str">
         <x:v>Diagramas de estados</x:v>
       </x:c>
-      <x:c r="C16" s="37" t="n">
-        <x:v>46324</x:v>
-      </x:c>
-      <x:c r="D16" s="37" t="n">
-        <x:v>46330</x:v>
+      <x:c r="C16" s="37" t="d">
+        <x:v>2026-10-31T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D16" s="37" t="d">
+        <x:v>2026-11-05T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="E16" s="9" t="n">
         <x:f>D16-C16+1</x:f>
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="F16" s="9" t="inlineStr">
         <x:is>
@@ -1115,11 +1226,11 @@
       <x:c r="B17" s="9" t="str">
         <x:v>Diagramas de sequência dos fluxos principais</x:v>
       </x:c>
-      <x:c r="C17" s="37" t="n">
-        <x:v>46328</x:v>
-      </x:c>
-      <x:c r="D17" s="37" t="n">
-        <x:v>46333</x:v>
+      <x:c r="C17" s="37" t="d">
+        <x:v>2026-11-03T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D17" s="37" t="d">
+        <x:v>2026-11-08T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="E17" s="9" t="n">
         <x:f>D17-C17+1</x:f>
@@ -1150,11 +1261,11 @@
       <x:c r="B18" s="12" t="str">
         <x:v>Definir arquitetura, tecnologias e organização da aplicação</x:v>
       </x:c>
-      <x:c r="C18" s="39" t="n">
-        <x:v>46328</x:v>
-      </x:c>
-      <x:c r="D18" s="39" t="n">
-        <x:v>46334</x:v>
+      <x:c r="C18" s="39" t="d">
+        <x:v>2026-11-02T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D18" s="39" t="d">
+        <x:v>2026-11-08T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="E18" s="12" t="n">
         <x:f>D18-C18+1</x:f>
@@ -1189,11 +1300,11 @@
       <x:c r="B19" s="12" t="str">
         <x:v>Diagrama de componentes</x:v>
       </x:c>
-      <x:c r="C19" s="39" t="n">
-        <x:v>46328</x:v>
-      </x:c>
-      <x:c r="D19" s="39" t="n">
-        <x:v>46334</x:v>
+      <x:c r="C19" s="39" t="d">
+        <x:v>2026-11-02T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D19" s="39" t="d">
+        <x:v>2026-11-08T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="E19" s="12" t="n">
         <x:f>D19-C19+1</x:f>
@@ -1228,15 +1339,15 @@
       <x:c r="B20" s="12" t="str">
         <x:v>Desenvolver/refinar protótipo das telas principais</x:v>
       </x:c>
-      <x:c r="C20" s="39" t="n">
-        <x:v>46329</x:v>
-      </x:c>
-      <x:c r="D20" s="39" t="n">
-        <x:v>46336</x:v>
+      <x:c r="C20" s="39" t="d">
+        <x:v>2026-11-04T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D20" s="39" t="d">
+        <x:v>2026-11-10T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="E20" s="12" t="n">
         <x:f>D20-C20+1</x:f>
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="F20" s="12" t="inlineStr">
         <x:is>
@@ -1265,11 +1376,11 @@
       <x:c r="B21" s="12" t="str">
         <x:v>Definir metodologia e cenários de validação</x:v>
       </x:c>
-      <x:c r="C21" s="39" t="n">
-        <x:v>46330</x:v>
-      </x:c>
-      <x:c r="D21" s="39" t="n">
-        <x:v>46336</x:v>
+      <x:c r="C21" s="39" t="d">
+        <x:v>2026-11-04T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D21" s="39" t="d">
+        <x:v>2026-11-10T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="E21" s="12" t="n">
         <x:f>D21-C21+1</x:f>
@@ -1296,15 +1407,15 @@
       <x:c r="B22" s="12" t="str">
         <x:v>Revisar documentação e consistência entre diagramas</x:v>
       </x:c>
-      <x:c r="C22" s="39" t="n">
-        <x:v>46335</x:v>
-      </x:c>
-      <x:c r="D22" s="39" t="n">
-        <x:v>46339</x:v>
+      <x:c r="C22" s="39" t="d">
+        <x:v>2026-11-09T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D22" s="39" t="d">
+        <x:v>2026-11-12T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="E22" s="12" t="n">
         <x:f>D22-C22+1</x:f>
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F22" s="12" t="str">
         <x:v>TCC1</x:v>
@@ -1327,11 +1438,11 @@
       <x:c r="B23" s="12" t="str">
         <x:v>Preparar apresentação, metodologia e pré-banca</x:v>
       </x:c>
-      <x:c r="C23" s="39" t="n">
-        <x:v>46337</x:v>
-      </x:c>
-      <x:c r="D23" s="39" t="n">
-        <x:v>46342</x:v>
+      <x:c r="C23" s="39" t="d">
+        <x:v>2026-11-11T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D23" s="39" t="d">
+        <x:v>2026-11-16T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="E23" s="12" t="n">
         <x:f>D23-C23+1</x:f>
@@ -2203,42 +2314,42 @@
       <x:c r="B4" s="43" t="str">
         <x:v>Finalizar e validar o fluxograma macro com o grupo</x:v>
       </x:c>
-      <x:c r="C4" s="35" t="n"/>
-      <x:c r="D4" s="35" t="n"/>
-      <x:c r="E4" s="35" t="n"/>
-      <x:c r="F4" s="36"/>
-      <x:c r="G4" s="36"/>
-      <x:c r="H4" s="35"/>
-      <x:c r="I4" s="35"/>
-      <x:c r="J4" s="35"/>
-      <x:c r="K4" s="35"/>
-      <x:c r="L4" s="35"/>
-      <x:c r="M4" s="35"/>
-      <x:c r="N4" s="35"/>
-      <x:c r="O4" s="35"/>
-      <x:c r="P4" s="35"/>
-      <x:c r="Q4" s="35"/>
-      <x:c r="R4" s="35"/>
-      <x:c r="S4" s="35"/>
-      <x:c r="T4" s="35"/>
-      <x:c r="U4" s="35"/>
-      <x:c r="V4" s="35"/>
-      <x:c r="W4" s="35"/>
-      <x:c r="X4" s="35"/>
-      <x:c r="Y4" s="35"/>
-      <x:c r="Z4" s="35"/>
-      <x:c r="AA4" s="35"/>
-      <x:c r="AB4" s="35"/>
-      <x:c r="AC4" s="35"/>
-      <x:c r="AD4" s="35"/>
-      <x:c r="AE4" s="35"/>
-      <x:c r="AF4" s="35"/>
-      <x:c r="AG4" s="35"/>
-      <x:c r="AH4" s="35"/>
-      <x:c r="AI4" s="35"/>
-      <x:c r="AJ4" s="35"/>
-      <x:c r="AK4" s="35"/>
-      <x:c r="AL4" s="35"/>
+      <x:c r="C4" s="48" t="n"/>
+      <x:c r="D4" s="48" t="n"/>
+      <x:c r="E4" s="48" t="n"/>
+      <x:c r="F4" s="48"/>
+      <x:c r="G4" s="48"/>
+      <x:c r="H4" s="48"/>
+      <x:c r="I4" s="48"/>
+      <x:c r="J4" s="48"/>
+      <x:c r="K4" s="48"/>
+      <x:c r="L4" s="48"/>
+      <x:c r="M4" s="48"/>
+      <x:c r="N4" s="48"/>
+      <x:c r="O4" s="48"/>
+      <x:c r="P4" s="48"/>
+      <x:c r="Q4" s="48"/>
+      <x:c r="R4" s="48"/>
+      <x:c r="S4" s="48"/>
+      <x:c r="T4" s="48"/>
+      <x:c r="U4" s="48"/>
+      <x:c r="V4" s="48"/>
+      <x:c r="W4" s="48"/>
+      <x:c r="X4" s="48"/>
+      <x:c r="Y4" s="48"/>
+      <x:c r="Z4" s="48"/>
+      <x:c r="AA4" s="48"/>
+      <x:c r="AB4" s="48"/>
+      <x:c r="AC4" s="48"/>
+      <x:c r="AD4" s="48"/>
+      <x:c r="AE4" s="48"/>
+      <x:c r="AF4" s="48"/>
+      <x:c r="AG4" s="48"/>
+      <x:c r="AH4" s="48"/>
+      <x:c r="AI4" s="48"/>
+      <x:c r="AJ4" s="48"/>
+      <x:c r="AK4" s="48"/>
+      <x:c r="AL4" s="48"/>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="42" t="str">
@@ -2247,42 +2358,42 @@
       <x:c r="B5" s="43" t="str">
         <x:v>Atualizar escopo, requisitos e regras de negócio</x:v>
       </x:c>
-      <x:c r="C5" s="35"/>
-      <x:c r="D5" s="35" t="n"/>
-      <x:c r="E5" s="35" t="n"/>
-      <x:c r="F5" s="36"/>
-      <x:c r="G5" s="36"/>
-      <x:c r="H5" s="35"/>
-      <x:c r="I5" s="35"/>
-      <x:c r="J5" s="35"/>
-      <x:c r="K5" s="35"/>
-      <x:c r="L5" s="35"/>
-      <x:c r="M5" s="35"/>
-      <x:c r="N5" s="35"/>
-      <x:c r="O5" s="35"/>
-      <x:c r="P5" s="35"/>
-      <x:c r="Q5" s="35"/>
-      <x:c r="R5" s="35"/>
-      <x:c r="S5" s="35"/>
-      <x:c r="T5" s="35"/>
-      <x:c r="U5" s="35"/>
-      <x:c r="V5" s="35"/>
-      <x:c r="W5" s="35"/>
-      <x:c r="X5" s="35"/>
-      <x:c r="Y5" s="35"/>
-      <x:c r="Z5" s="35"/>
-      <x:c r="AA5" s="35"/>
-      <x:c r="AB5" s="35"/>
-      <x:c r="AC5" s="35"/>
-      <x:c r="AD5" s="35"/>
-      <x:c r="AE5" s="35"/>
-      <x:c r="AF5" s="35"/>
-      <x:c r="AG5" s="35"/>
-      <x:c r="AH5" s="35"/>
-      <x:c r="AI5" s="35"/>
-      <x:c r="AJ5" s="35"/>
-      <x:c r="AK5" s="35"/>
-      <x:c r="AL5" s="35"/>
+      <x:c r="C5" s="48"/>
+      <x:c r="D5" s="48" t="n"/>
+      <x:c r="E5" s="48" t="n"/>
+      <x:c r="F5" s="48"/>
+      <x:c r="G5" s="48"/>
+      <x:c r="H5" s="48"/>
+      <x:c r="I5" s="48"/>
+      <x:c r="J5" s="48"/>
+      <x:c r="K5" s="48"/>
+      <x:c r="L5" s="48"/>
+      <x:c r="M5" s="48"/>
+      <x:c r="N5" s="48"/>
+      <x:c r="O5" s="48"/>
+      <x:c r="P5" s="48"/>
+      <x:c r="Q5" s="48"/>
+      <x:c r="R5" s="48"/>
+      <x:c r="S5" s="48"/>
+      <x:c r="T5" s="48"/>
+      <x:c r="U5" s="48"/>
+      <x:c r="V5" s="48"/>
+      <x:c r="W5" s="48"/>
+      <x:c r="X5" s="48"/>
+      <x:c r="Y5" s="48"/>
+      <x:c r="Z5" s="48"/>
+      <x:c r="AA5" s="48"/>
+      <x:c r="AB5" s="48"/>
+      <x:c r="AC5" s="48"/>
+      <x:c r="AD5" s="48"/>
+      <x:c r="AE5" s="48"/>
+      <x:c r="AF5" s="48"/>
+      <x:c r="AG5" s="48"/>
+      <x:c r="AH5" s="48"/>
+      <x:c r="AI5" s="48"/>
+      <x:c r="AJ5" s="48"/>
+      <x:c r="AK5" s="48"/>
+      <x:c r="AL5" s="48"/>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="42" t="str">
@@ -2291,42 +2402,42 @@
       <x:c r="B6" s="43" t="str">
         <x:v>Finalizar atores, casos de uso e responsabilidades</x:v>
       </x:c>
-      <x:c r="C6" s="35"/>
-      <x:c r="D6" s="35"/>
-      <x:c r="E6" s="35" t="n"/>
-      <x:c r="F6" s="35" t="n"/>
-      <x:c r="G6" s="36"/>
-      <x:c r="H6" s="36"/>
-      <x:c r="I6" s="35"/>
-      <x:c r="J6" s="35"/>
-      <x:c r="K6" s="35"/>
-      <x:c r="L6" s="35"/>
-      <x:c r="M6" s="35"/>
-      <x:c r="N6" s="35"/>
-      <x:c r="O6" s="35"/>
-      <x:c r="P6" s="35"/>
-      <x:c r="Q6" s="35"/>
-      <x:c r="R6" s="35"/>
-      <x:c r="S6" s="35"/>
-      <x:c r="T6" s="35"/>
-      <x:c r="U6" s="35"/>
-      <x:c r="V6" s="35"/>
-      <x:c r="W6" s="35"/>
-      <x:c r="X6" s="35"/>
-      <x:c r="Y6" s="35"/>
-      <x:c r="Z6" s="35"/>
-      <x:c r="AA6" s="35"/>
-      <x:c r="AB6" s="35"/>
-      <x:c r="AC6" s="35"/>
-      <x:c r="AD6" s="35"/>
-      <x:c r="AE6" s="35"/>
-      <x:c r="AF6" s="35"/>
-      <x:c r="AG6" s="35"/>
-      <x:c r="AH6" s="35"/>
-      <x:c r="AI6" s="35"/>
-      <x:c r="AJ6" s="35"/>
-      <x:c r="AK6" s="35"/>
-      <x:c r="AL6" s="35"/>
+      <x:c r="C6" s="48"/>
+      <x:c r="D6" s="48"/>
+      <x:c r="E6" s="48" t="n"/>
+      <x:c r="F6" s="48" t="n"/>
+      <x:c r="G6" s="48"/>
+      <x:c r="H6" s="48"/>
+      <x:c r="I6" s="48"/>
+      <x:c r="J6" s="48"/>
+      <x:c r="K6" s="48"/>
+      <x:c r="L6" s="48"/>
+      <x:c r="M6" s="48"/>
+      <x:c r="N6" s="48"/>
+      <x:c r="O6" s="48"/>
+      <x:c r="P6" s="48"/>
+      <x:c r="Q6" s="48"/>
+      <x:c r="R6" s="48"/>
+      <x:c r="S6" s="48"/>
+      <x:c r="T6" s="48"/>
+      <x:c r="U6" s="48"/>
+      <x:c r="V6" s="48"/>
+      <x:c r="W6" s="48"/>
+      <x:c r="X6" s="48"/>
+      <x:c r="Y6" s="48"/>
+      <x:c r="Z6" s="48"/>
+      <x:c r="AA6" s="48"/>
+      <x:c r="AB6" s="48"/>
+      <x:c r="AC6" s="48"/>
+      <x:c r="AD6" s="48"/>
+      <x:c r="AE6" s="48"/>
+      <x:c r="AF6" s="48"/>
+      <x:c r="AG6" s="48"/>
+      <x:c r="AH6" s="48"/>
+      <x:c r="AI6" s="48"/>
+      <x:c r="AJ6" s="48"/>
+      <x:c r="AK6" s="48"/>
+      <x:c r="AL6" s="48"/>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="42" t="str">
@@ -2335,42 +2446,42 @@
       <x:c r="B7" s="43" t="str">
         <x:v>Diagrama de casos de uso + descrições principais</x:v>
       </x:c>
-      <x:c r="C7" s="35"/>
-      <x:c r="D7" s="35"/>
-      <x:c r="E7" s="35"/>
-      <x:c r="F7" s="35" t="n"/>
-      <x:c r="G7" s="36" t="n"/>
-      <x:c r="H7" s="36"/>
-      <x:c r="I7" s="35"/>
-      <x:c r="J7" s="35"/>
-      <x:c r="K7" s="35"/>
-      <x:c r="L7" s="35"/>
-      <x:c r="M7" s="35"/>
-      <x:c r="N7" s="35"/>
-      <x:c r="O7" s="35"/>
-      <x:c r="P7" s="35"/>
-      <x:c r="Q7" s="35"/>
-      <x:c r="R7" s="35"/>
-      <x:c r="S7" s="35"/>
-      <x:c r="T7" s="35"/>
-      <x:c r="U7" s="35"/>
-      <x:c r="V7" s="35"/>
-      <x:c r="W7" s="35"/>
-      <x:c r="X7" s="35"/>
-      <x:c r="Y7" s="35"/>
-      <x:c r="Z7" s="35"/>
-      <x:c r="AA7" s="35"/>
-      <x:c r="AB7" s="35"/>
-      <x:c r="AC7" s="35"/>
-      <x:c r="AD7" s="35"/>
-      <x:c r="AE7" s="35"/>
-      <x:c r="AF7" s="35"/>
-      <x:c r="AG7" s="35"/>
-      <x:c r="AH7" s="35"/>
-      <x:c r="AI7" s="35"/>
-      <x:c r="AJ7" s="35"/>
-      <x:c r="AK7" s="35"/>
-      <x:c r="AL7" s="35"/>
+      <x:c r="C7" s="48"/>
+      <x:c r="D7" s="48"/>
+      <x:c r="E7" s="48"/>
+      <x:c r="F7" s="48" t="n"/>
+      <x:c r="G7" s="48" t="n"/>
+      <x:c r="H7" s="48"/>
+      <x:c r="I7" s="48"/>
+      <x:c r="J7" s="48"/>
+      <x:c r="K7" s="48"/>
+      <x:c r="L7" s="48"/>
+      <x:c r="M7" s="48"/>
+      <x:c r="N7" s="48"/>
+      <x:c r="O7" s="48"/>
+      <x:c r="P7" s="48"/>
+      <x:c r="Q7" s="48"/>
+      <x:c r="R7" s="48"/>
+      <x:c r="S7" s="48"/>
+      <x:c r="T7" s="48"/>
+      <x:c r="U7" s="48"/>
+      <x:c r="V7" s="48"/>
+      <x:c r="W7" s="48"/>
+      <x:c r="X7" s="48"/>
+      <x:c r="Y7" s="48"/>
+      <x:c r="Z7" s="48"/>
+      <x:c r="AA7" s="48"/>
+      <x:c r="AB7" s="48"/>
+      <x:c r="AC7" s="48"/>
+      <x:c r="AD7" s="48"/>
+      <x:c r="AE7" s="48"/>
+      <x:c r="AF7" s="48"/>
+      <x:c r="AG7" s="48"/>
+      <x:c r="AH7" s="48"/>
+      <x:c r="AI7" s="48"/>
+      <x:c r="AJ7" s="48"/>
+      <x:c r="AK7" s="48"/>
+      <x:c r="AL7" s="48"/>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="42" t="str">
@@ -2379,42 +2490,42 @@
       <x:c r="B8" s="43" t="str">
         <x:v>Diagrama de classes de domínio</x:v>
       </x:c>
-      <x:c r="C8" s="35"/>
-      <x:c r="D8" s="35"/>
-      <x:c r="E8" s="35"/>
-      <x:c r="F8" s="35"/>
-      <x:c r="G8" s="35"/>
-      <x:c r="H8" s="36"/>
-      <x:c r="I8" s="35"/>
-      <x:c r="J8" s="35"/>
-      <x:c r="K8" s="35"/>
-      <x:c r="L8" s="35"/>
-      <x:c r="M8" s="35"/>
-      <x:c r="N8" s="35"/>
-      <x:c r="O8" s="35"/>
-      <x:c r="P8" s="35"/>
-      <x:c r="Q8" s="35"/>
-      <x:c r="R8" s="35"/>
-      <x:c r="S8" s="35"/>
-      <x:c r="T8" s="35"/>
-      <x:c r="U8" s="35"/>
-      <x:c r="V8" s="35"/>
-      <x:c r="W8" s="35"/>
-      <x:c r="X8" s="35"/>
-      <x:c r="Y8" s="35"/>
-      <x:c r="Z8" s="35"/>
-      <x:c r="AA8" s="35"/>
-      <x:c r="AB8" s="35"/>
-      <x:c r="AC8" s="35"/>
-      <x:c r="AD8" s="35"/>
-      <x:c r="AE8" s="35"/>
-      <x:c r="AF8" s="35"/>
-      <x:c r="AG8" s="35"/>
-      <x:c r="AH8" s="35"/>
-      <x:c r="AI8" s="35"/>
-      <x:c r="AJ8" s="35"/>
-      <x:c r="AK8" s="35"/>
-      <x:c r="AL8" s="35"/>
+      <x:c r="C8" s="48"/>
+      <x:c r="D8" s="48"/>
+      <x:c r="E8" s="48"/>
+      <x:c r="F8" s="48"/>
+      <x:c r="G8" s="48"/>
+      <x:c r="H8" s="48"/>
+      <x:c r="I8" s="48"/>
+      <x:c r="J8" s="48"/>
+      <x:c r="K8" s="48"/>
+      <x:c r="L8" s="48"/>
+      <x:c r="M8" s="48"/>
+      <x:c r="N8" s="48"/>
+      <x:c r="O8" s="48"/>
+      <x:c r="P8" s="48"/>
+      <x:c r="Q8" s="48"/>
+      <x:c r="R8" s="48"/>
+      <x:c r="S8" s="48"/>
+      <x:c r="T8" s="48"/>
+      <x:c r="U8" s="48"/>
+      <x:c r="V8" s="48"/>
+      <x:c r="W8" s="48"/>
+      <x:c r="X8" s="48"/>
+      <x:c r="Y8" s="48"/>
+      <x:c r="Z8" s="48"/>
+      <x:c r="AA8" s="48"/>
+      <x:c r="AB8" s="48"/>
+      <x:c r="AC8" s="48"/>
+      <x:c r="AD8" s="48"/>
+      <x:c r="AE8" s="48"/>
+      <x:c r="AF8" s="48"/>
+      <x:c r="AG8" s="48"/>
+      <x:c r="AH8" s="48"/>
+      <x:c r="AI8" s="48"/>
+      <x:c r="AJ8" s="48"/>
+      <x:c r="AK8" s="48"/>
+      <x:c r="AL8" s="48"/>
     </x:row>
     <x:row r="9" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A9" s="44" t="str">
@@ -2423,42 +2534,42 @@
       <x:c r="B9" s="45" t="str">
         <x:v>DER e modelagem do banco de dados</x:v>
       </x:c>
-      <x:c r="C9" s="35"/>
-      <x:c r="D9" s="35"/>
-      <x:c r="E9" s="35"/>
-      <x:c r="F9" s="35"/>
-      <x:c r="G9" s="35"/>
-      <x:c r="H9" s="38" t="n"/>
-      <x:c r="I9" s="38" t="n"/>
-      <x:c r="J9" s="35"/>
-      <x:c r="K9" s="35"/>
-      <x:c r="L9" s="35"/>
-      <x:c r="M9" s="35"/>
-      <x:c r="N9" s="35"/>
-      <x:c r="O9" s="35"/>
-      <x:c r="P9" s="35"/>
-      <x:c r="Q9" s="35"/>
-      <x:c r="R9" s="35"/>
-      <x:c r="S9" s="35"/>
-      <x:c r="T9" s="35"/>
-      <x:c r="U9" s="35"/>
-      <x:c r="V9" s="35"/>
-      <x:c r="W9" s="35"/>
-      <x:c r="X9" s="35"/>
-      <x:c r="Y9" s="35"/>
-      <x:c r="Z9" s="35"/>
-      <x:c r="AA9" s="35"/>
-      <x:c r="AB9" s="35"/>
-      <x:c r="AC9" s="35"/>
-      <x:c r="AD9" s="35"/>
-      <x:c r="AE9" s="35"/>
-      <x:c r="AF9" s="35"/>
-      <x:c r="AG9" s="35"/>
-      <x:c r="AH9" s="35"/>
-      <x:c r="AI9" s="35"/>
-      <x:c r="AJ9" s="35"/>
-      <x:c r="AK9" s="35"/>
-      <x:c r="AL9" s="35"/>
+      <x:c r="C9" s="48"/>
+      <x:c r="D9" s="48"/>
+      <x:c r="E9" s="48"/>
+      <x:c r="F9" s="48"/>
+      <x:c r="G9" s="48"/>
+      <x:c r="H9" s="48" t="n"/>
+      <x:c r="I9" s="48" t="n"/>
+      <x:c r="J9" s="48"/>
+      <x:c r="K9" s="48"/>
+      <x:c r="L9" s="48"/>
+      <x:c r="M9" s="48"/>
+      <x:c r="N9" s="48"/>
+      <x:c r="O9" s="48"/>
+      <x:c r="P9" s="48"/>
+      <x:c r="Q9" s="48"/>
+      <x:c r="R9" s="48"/>
+      <x:c r="S9" s="48"/>
+      <x:c r="T9" s="48"/>
+      <x:c r="U9" s="48"/>
+      <x:c r="V9" s="48"/>
+      <x:c r="W9" s="48"/>
+      <x:c r="X9" s="48"/>
+      <x:c r="Y9" s="48"/>
+      <x:c r="Z9" s="48"/>
+      <x:c r="AA9" s="48"/>
+      <x:c r="AB9" s="48"/>
+      <x:c r="AC9" s="48"/>
+      <x:c r="AD9" s="48"/>
+      <x:c r="AE9" s="48"/>
+      <x:c r="AF9" s="48"/>
+      <x:c r="AG9" s="48"/>
+      <x:c r="AH9" s="48"/>
+      <x:c r="AI9" s="48"/>
+      <x:c r="AJ9" s="48"/>
+      <x:c r="AK9" s="48"/>
+      <x:c r="AL9" s="48"/>
     </x:row>
     <x:row r="10" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A10" s="44" t="str">
@@ -2467,42 +2578,42 @@
       <x:c r="B10" s="45" t="str">
         <x:v>Diagramas de atividades dos fluxos principais</x:v>
       </x:c>
-      <x:c r="C10" s="35"/>
-      <x:c r="D10" s="35"/>
-      <x:c r="E10" s="35"/>
-      <x:c r="F10" s="35"/>
-      <x:c r="G10" s="35"/>
-      <x:c r="H10" s="35"/>
-      <x:c r="I10" s="38" t="n"/>
-      <x:c r="J10" s="35"/>
-      <x:c r="K10" s="35"/>
-      <x:c r="L10" s="35"/>
-      <x:c r="M10" s="35"/>
-      <x:c r="N10" s="35"/>
-      <x:c r="O10" s="35"/>
-      <x:c r="P10" s="35"/>
-      <x:c r="Q10" s="35"/>
-      <x:c r="R10" s="35"/>
-      <x:c r="S10" s="35"/>
-      <x:c r="T10" s="35"/>
-      <x:c r="U10" s="35"/>
-      <x:c r="V10" s="35"/>
-      <x:c r="W10" s="35"/>
-      <x:c r="X10" s="35"/>
-      <x:c r="Y10" s="35"/>
-      <x:c r="Z10" s="35"/>
-      <x:c r="AA10" s="35"/>
-      <x:c r="AB10" s="35"/>
-      <x:c r="AC10" s="35"/>
-      <x:c r="AD10" s="35"/>
-      <x:c r="AE10" s="35"/>
-      <x:c r="AF10" s="35"/>
-      <x:c r="AG10" s="35"/>
-      <x:c r="AH10" s="35"/>
-      <x:c r="AI10" s="35"/>
-      <x:c r="AJ10" s="35"/>
-      <x:c r="AK10" s="35"/>
-      <x:c r="AL10" s="35"/>
+      <x:c r="C10" s="48"/>
+      <x:c r="D10" s="48"/>
+      <x:c r="E10" s="48"/>
+      <x:c r="F10" s="48"/>
+      <x:c r="G10" s="48"/>
+      <x:c r="H10" s="48"/>
+      <x:c r="I10" s="48" t="n"/>
+      <x:c r="J10" s="48"/>
+      <x:c r="K10" s="48"/>
+      <x:c r="L10" s="48"/>
+      <x:c r="M10" s="48"/>
+      <x:c r="N10" s="48"/>
+      <x:c r="O10" s="48"/>
+      <x:c r="P10" s="48"/>
+      <x:c r="Q10" s="48"/>
+      <x:c r="R10" s="48"/>
+      <x:c r="S10" s="48"/>
+      <x:c r="T10" s="48"/>
+      <x:c r="U10" s="48"/>
+      <x:c r="V10" s="48"/>
+      <x:c r="W10" s="48"/>
+      <x:c r="X10" s="48"/>
+      <x:c r="Y10" s="48"/>
+      <x:c r="Z10" s="48"/>
+      <x:c r="AA10" s="48"/>
+      <x:c r="AB10" s="48"/>
+      <x:c r="AC10" s="48"/>
+      <x:c r="AD10" s="48"/>
+      <x:c r="AE10" s="48"/>
+      <x:c r="AF10" s="48"/>
+      <x:c r="AG10" s="48"/>
+      <x:c r="AH10" s="48"/>
+      <x:c r="AI10" s="48"/>
+      <x:c r="AJ10" s="48"/>
+      <x:c r="AK10" s="48"/>
+      <x:c r="AL10" s="48"/>
     </x:row>
     <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A11" s="44" t="str">
@@ -2511,42 +2622,42 @@
       <x:c r="B11" s="45" t="str">
         <x:v>Diagramas de estados</x:v>
       </x:c>
-      <x:c r="C11" s="35"/>
-      <x:c r="D11" s="35"/>
-      <x:c r="E11" s="35"/>
-      <x:c r="F11" s="35"/>
-      <x:c r="G11" s="35"/>
-      <x:c r="H11" s="35"/>
-      <x:c r="I11" s="38" t="n"/>
-      <x:c r="J11" s="35" t="n"/>
-      <x:c r="K11" s="35"/>
-      <x:c r="L11" s="35"/>
-      <x:c r="M11" s="35"/>
-      <x:c r="N11" s="35"/>
-      <x:c r="O11" s="35"/>
-      <x:c r="P11" s="35"/>
-      <x:c r="Q11" s="35"/>
-      <x:c r="R11" s="35"/>
-      <x:c r="S11" s="35"/>
-      <x:c r="T11" s="35"/>
-      <x:c r="U11" s="35"/>
-      <x:c r="V11" s="35"/>
-      <x:c r="W11" s="35"/>
-      <x:c r="X11" s="35"/>
-      <x:c r="Y11" s="35"/>
-      <x:c r="Z11" s="35"/>
-      <x:c r="AA11" s="35"/>
-      <x:c r="AB11" s="35"/>
-      <x:c r="AC11" s="35"/>
-      <x:c r="AD11" s="35"/>
-      <x:c r="AE11" s="35"/>
-      <x:c r="AF11" s="35"/>
-      <x:c r="AG11" s="35"/>
-      <x:c r="AH11" s="35"/>
-      <x:c r="AI11" s="35"/>
-      <x:c r="AJ11" s="35"/>
-      <x:c r="AK11" s="35"/>
-      <x:c r="AL11" s="35"/>
+      <x:c r="C11" s="48"/>
+      <x:c r="D11" s="48"/>
+      <x:c r="E11" s="48"/>
+      <x:c r="F11" s="48"/>
+      <x:c r="G11" s="48"/>
+      <x:c r="H11" s="48"/>
+      <x:c r="I11" s="48" t="n"/>
+      <x:c r="J11" s="48" t="n"/>
+      <x:c r="K11" s="48"/>
+      <x:c r="L11" s="48"/>
+      <x:c r="M11" s="48"/>
+      <x:c r="N11" s="48"/>
+      <x:c r="O11" s="48"/>
+      <x:c r="P11" s="48"/>
+      <x:c r="Q11" s="48"/>
+      <x:c r="R11" s="48"/>
+      <x:c r="S11" s="48"/>
+      <x:c r="T11" s="48"/>
+      <x:c r="U11" s="48"/>
+      <x:c r="V11" s="48"/>
+      <x:c r="W11" s="48"/>
+      <x:c r="X11" s="48"/>
+      <x:c r="Y11" s="48"/>
+      <x:c r="Z11" s="48"/>
+      <x:c r="AA11" s="48"/>
+      <x:c r="AB11" s="48"/>
+      <x:c r="AC11" s="48"/>
+      <x:c r="AD11" s="48"/>
+      <x:c r="AE11" s="48"/>
+      <x:c r="AF11" s="48"/>
+      <x:c r="AG11" s="48"/>
+      <x:c r="AH11" s="48"/>
+      <x:c r="AI11" s="48"/>
+      <x:c r="AJ11" s="48"/>
+      <x:c r="AK11" s="48"/>
+      <x:c r="AL11" s="48"/>
     </x:row>
     <x:row r="12" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A12" s="44" t="str">
@@ -2555,42 +2666,42 @@
       <x:c r="B12" s="45" t="str">
         <x:v>Diagramas de sequência dos fluxos principais</x:v>
       </x:c>
-      <x:c r="C12" s="35"/>
-      <x:c r="D12" s="35"/>
-      <x:c r="E12" s="35"/>
-      <x:c r="F12" s="35"/>
-      <x:c r="G12" s="35"/>
-      <x:c r="H12" s="35"/>
-      <x:c r="I12" s="38"/>
-      <x:c r="J12" s="38"/>
-      <x:c r="K12" s="35"/>
-      <x:c r="L12" s="35"/>
-      <x:c r="M12" s="35"/>
-      <x:c r="N12" s="35"/>
-      <x:c r="O12" s="35"/>
-      <x:c r="P12" s="35"/>
-      <x:c r="Q12" s="35"/>
-      <x:c r="R12" s="35"/>
-      <x:c r="S12" s="35"/>
-      <x:c r="T12" s="35"/>
-      <x:c r="U12" s="35"/>
-      <x:c r="V12" s="35"/>
-      <x:c r="W12" s="35"/>
-      <x:c r="X12" s="35"/>
-      <x:c r="Y12" s="35"/>
-      <x:c r="Z12" s="35"/>
-      <x:c r="AA12" s="35"/>
-      <x:c r="AB12" s="35"/>
-      <x:c r="AC12" s="35"/>
-      <x:c r="AD12" s="35"/>
-      <x:c r="AE12" s="35"/>
-      <x:c r="AF12" s="35"/>
-      <x:c r="AG12" s="35"/>
-      <x:c r="AH12" s="35"/>
-      <x:c r="AI12" s="35"/>
-      <x:c r="AJ12" s="35"/>
-      <x:c r="AK12" s="35"/>
-      <x:c r="AL12" s="35"/>
+      <x:c r="C12" s="48"/>
+      <x:c r="D12" s="48"/>
+      <x:c r="E12" s="48"/>
+      <x:c r="F12" s="48"/>
+      <x:c r="G12" s="48"/>
+      <x:c r="H12" s="48"/>
+      <x:c r="I12" s="48"/>
+      <x:c r="J12" s="48"/>
+      <x:c r="K12" s="48"/>
+      <x:c r="L12" s="48"/>
+      <x:c r="M12" s="48"/>
+      <x:c r="N12" s="48"/>
+      <x:c r="O12" s="48"/>
+      <x:c r="P12" s="48"/>
+      <x:c r="Q12" s="48"/>
+      <x:c r="R12" s="48"/>
+      <x:c r="S12" s="48"/>
+      <x:c r="T12" s="48"/>
+      <x:c r="U12" s="48"/>
+      <x:c r="V12" s="48"/>
+      <x:c r="W12" s="48"/>
+      <x:c r="X12" s="48"/>
+      <x:c r="Y12" s="48"/>
+      <x:c r="Z12" s="48"/>
+      <x:c r="AA12" s="48"/>
+      <x:c r="AB12" s="48"/>
+      <x:c r="AC12" s="48"/>
+      <x:c r="AD12" s="48"/>
+      <x:c r="AE12" s="48"/>
+      <x:c r="AF12" s="48"/>
+      <x:c r="AG12" s="48"/>
+      <x:c r="AH12" s="48"/>
+      <x:c r="AI12" s="48"/>
+      <x:c r="AJ12" s="48"/>
+      <x:c r="AK12" s="48"/>
+      <x:c r="AL12" s="48"/>
     </x:row>
     <x:row r="13" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A13" s="46" t="str">
@@ -2599,42 +2710,42 @@
       <x:c r="B13" s="47" t="str">
         <x:v>Definir arquitetura, tecnologias e organização da aplicação</x:v>
       </x:c>
-      <x:c r="C13" s="35"/>
-      <x:c r="D13" s="35"/>
-      <x:c r="E13" s="35"/>
-      <x:c r="F13" s="35"/>
-      <x:c r="G13" s="35"/>
-      <x:c r="H13" s="35"/>
-      <x:c r="I13" s="40" t="n"/>
-      <x:c r="J13" s="40" t="n"/>
-      <x:c r="K13" s="35"/>
-      <x:c r="L13" s="35"/>
-      <x:c r="M13" s="35"/>
-      <x:c r="N13" s="35"/>
-      <x:c r="O13" s="35"/>
-      <x:c r="P13" s="35"/>
-      <x:c r="Q13" s="35"/>
-      <x:c r="R13" s="35"/>
-      <x:c r="S13" s="35"/>
-      <x:c r="T13" s="35"/>
-      <x:c r="U13" s="35"/>
-      <x:c r="V13" s="35"/>
-      <x:c r="W13" s="35"/>
-      <x:c r="X13" s="35"/>
-      <x:c r="Y13" s="35"/>
-      <x:c r="Z13" s="35"/>
-      <x:c r="AA13" s="35"/>
-      <x:c r="AB13" s="35"/>
-      <x:c r="AC13" s="35"/>
-      <x:c r="AD13" s="35"/>
-      <x:c r="AE13" s="35"/>
-      <x:c r="AF13" s="35"/>
-      <x:c r="AG13" s="35"/>
-      <x:c r="AH13" s="35"/>
-      <x:c r="AI13" s="35"/>
-      <x:c r="AJ13" s="35"/>
-      <x:c r="AK13" s="35"/>
-      <x:c r="AL13" s="35"/>
+      <x:c r="C13" s="48"/>
+      <x:c r="D13" s="48"/>
+      <x:c r="E13" s="48"/>
+      <x:c r="F13" s="48"/>
+      <x:c r="G13" s="48"/>
+      <x:c r="H13" s="48"/>
+      <x:c r="I13" s="48" t="n"/>
+      <x:c r="J13" s="48" t="n"/>
+      <x:c r="K13" s="48"/>
+      <x:c r="L13" s="48"/>
+      <x:c r="M13" s="48"/>
+      <x:c r="N13" s="48"/>
+      <x:c r="O13" s="48"/>
+      <x:c r="P13" s="48"/>
+      <x:c r="Q13" s="48"/>
+      <x:c r="R13" s="48"/>
+      <x:c r="S13" s="48"/>
+      <x:c r="T13" s="48"/>
+      <x:c r="U13" s="48"/>
+      <x:c r="V13" s="48"/>
+      <x:c r="W13" s="48"/>
+      <x:c r="X13" s="48"/>
+      <x:c r="Y13" s="48"/>
+      <x:c r="Z13" s="48"/>
+      <x:c r="AA13" s="48"/>
+      <x:c r="AB13" s="48"/>
+      <x:c r="AC13" s="48"/>
+      <x:c r="AD13" s="48"/>
+      <x:c r="AE13" s="48"/>
+      <x:c r="AF13" s="48"/>
+      <x:c r="AG13" s="48"/>
+      <x:c r="AH13" s="48"/>
+      <x:c r="AI13" s="48"/>
+      <x:c r="AJ13" s="48"/>
+      <x:c r="AK13" s="48"/>
+      <x:c r="AL13" s="48"/>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="46" t="str">
@@ -2643,42 +2754,42 @@
       <x:c r="B14" s="47" t="str">
         <x:v>Diagrama de componentes</x:v>
       </x:c>
-      <x:c r="C14" s="35"/>
-      <x:c r="D14" s="35"/>
-      <x:c r="E14" s="35"/>
-      <x:c r="F14" s="35"/>
-      <x:c r="G14" s="35"/>
-      <x:c r="H14" s="35"/>
-      <x:c r="I14" s="40" t="n"/>
-      <x:c r="J14" s="40" t="n"/>
-      <x:c r="K14" s="35"/>
-      <x:c r="L14" s="35"/>
-      <x:c r="M14" s="35"/>
-      <x:c r="N14" s="35"/>
-      <x:c r="O14" s="35"/>
-      <x:c r="P14" s="35"/>
-      <x:c r="Q14" s="35"/>
-      <x:c r="R14" s="35"/>
-      <x:c r="S14" s="35"/>
-      <x:c r="T14" s="35"/>
-      <x:c r="U14" s="35"/>
-      <x:c r="V14" s="35"/>
-      <x:c r="W14" s="35"/>
-      <x:c r="X14" s="35"/>
-      <x:c r="Y14" s="35"/>
-      <x:c r="Z14" s="35"/>
-      <x:c r="AA14" s="35"/>
-      <x:c r="AB14" s="35"/>
-      <x:c r="AC14" s="35"/>
-      <x:c r="AD14" s="35"/>
-      <x:c r="AE14" s="35"/>
-      <x:c r="AF14" s="35"/>
-      <x:c r="AG14" s="35"/>
-      <x:c r="AH14" s="35"/>
-      <x:c r="AI14" s="35"/>
-      <x:c r="AJ14" s="35"/>
-      <x:c r="AK14" s="35"/>
-      <x:c r="AL14" s="35"/>
+      <x:c r="C14" s="48"/>
+      <x:c r="D14" s="48"/>
+      <x:c r="E14" s="48"/>
+      <x:c r="F14" s="48"/>
+      <x:c r="G14" s="48"/>
+      <x:c r="H14" s="48"/>
+      <x:c r="I14" s="48" t="n"/>
+      <x:c r="J14" s="48" t="n"/>
+      <x:c r="K14" s="48"/>
+      <x:c r="L14" s="48"/>
+      <x:c r="M14" s="48"/>
+      <x:c r="N14" s="48"/>
+      <x:c r="O14" s="48"/>
+      <x:c r="P14" s="48"/>
+      <x:c r="Q14" s="48"/>
+      <x:c r="R14" s="48"/>
+      <x:c r="S14" s="48"/>
+      <x:c r="T14" s="48"/>
+      <x:c r="U14" s="48"/>
+      <x:c r="V14" s="48"/>
+      <x:c r="W14" s="48"/>
+      <x:c r="X14" s="48"/>
+      <x:c r="Y14" s="48"/>
+      <x:c r="Z14" s="48"/>
+      <x:c r="AA14" s="48"/>
+      <x:c r="AB14" s="48"/>
+      <x:c r="AC14" s="48"/>
+      <x:c r="AD14" s="48"/>
+      <x:c r="AE14" s="48"/>
+      <x:c r="AF14" s="48"/>
+      <x:c r="AG14" s="48"/>
+      <x:c r="AH14" s="48"/>
+      <x:c r="AI14" s="48"/>
+      <x:c r="AJ14" s="48"/>
+      <x:c r="AK14" s="48"/>
+      <x:c r="AL14" s="48"/>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="46" t="str">
@@ -2687,42 +2798,42 @@
       <x:c r="B15" s="47" t="str">
         <x:v>Desenvolver/refinar protótipo das telas principais</x:v>
       </x:c>
-      <x:c r="C15" s="35"/>
-      <x:c r="D15" s="35"/>
-      <x:c r="E15" s="35"/>
-      <x:c r="F15" s="35"/>
-      <x:c r="G15" s="35"/>
-      <x:c r="H15" s="35"/>
-      <x:c r="I15" s="40"/>
-      <x:c r="J15" s="40" t="n"/>
-      <x:c r="K15" s="35"/>
-      <x:c r="L15" s="35"/>
-      <x:c r="M15" s="35"/>
-      <x:c r="N15" s="35"/>
-      <x:c r="O15" s="35"/>
-      <x:c r="P15" s="35"/>
-      <x:c r="Q15" s="35"/>
-      <x:c r="R15" s="35"/>
-      <x:c r="S15" s="35"/>
-      <x:c r="T15" s="35"/>
-      <x:c r="U15" s="35"/>
-      <x:c r="V15" s="35"/>
-      <x:c r="W15" s="35"/>
-      <x:c r="X15" s="35"/>
-      <x:c r="Y15" s="35"/>
-      <x:c r="Z15" s="35"/>
-      <x:c r="AA15" s="35"/>
-      <x:c r="AB15" s="35"/>
-      <x:c r="AC15" s="35"/>
-      <x:c r="AD15" s="35"/>
-      <x:c r="AE15" s="35"/>
-      <x:c r="AF15" s="35"/>
-      <x:c r="AG15" s="35"/>
-      <x:c r="AH15" s="35"/>
-      <x:c r="AI15" s="35"/>
-      <x:c r="AJ15" s="35"/>
-      <x:c r="AK15" s="35"/>
-      <x:c r="AL15" s="35"/>
+      <x:c r="C15" s="48"/>
+      <x:c r="D15" s="48"/>
+      <x:c r="E15" s="48"/>
+      <x:c r="F15" s="48"/>
+      <x:c r="G15" s="48"/>
+      <x:c r="H15" s="48"/>
+      <x:c r="I15" s="48"/>
+      <x:c r="J15" s="48" t="n"/>
+      <x:c r="K15" s="48"/>
+      <x:c r="L15" s="48"/>
+      <x:c r="M15" s="48"/>
+      <x:c r="N15" s="48"/>
+      <x:c r="O15" s="48"/>
+      <x:c r="P15" s="48"/>
+      <x:c r="Q15" s="48"/>
+      <x:c r="R15" s="48"/>
+      <x:c r="S15" s="48"/>
+      <x:c r="T15" s="48"/>
+      <x:c r="U15" s="48"/>
+      <x:c r="V15" s="48"/>
+      <x:c r="W15" s="48"/>
+      <x:c r="X15" s="48"/>
+      <x:c r="Y15" s="48"/>
+      <x:c r="Z15" s="48"/>
+      <x:c r="AA15" s="48"/>
+      <x:c r="AB15" s="48"/>
+      <x:c r="AC15" s="48"/>
+      <x:c r="AD15" s="48"/>
+      <x:c r="AE15" s="48"/>
+      <x:c r="AF15" s="48"/>
+      <x:c r="AG15" s="48"/>
+      <x:c r="AH15" s="48"/>
+      <x:c r="AI15" s="48"/>
+      <x:c r="AJ15" s="48"/>
+      <x:c r="AK15" s="48"/>
+      <x:c r="AL15" s="48"/>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="46" t="str">
@@ -2731,42 +2842,42 @@
       <x:c r="B16" s="47" t="str">
         <x:v>Definir metodologia e cenários de validação</x:v>
       </x:c>
-      <x:c r="C16" s="35"/>
-      <x:c r="D16" s="35"/>
-      <x:c r="E16" s="35"/>
-      <x:c r="F16" s="35"/>
-      <x:c r="G16" s="35"/>
-      <x:c r="H16" s="35"/>
-      <x:c r="I16" s="40"/>
-      <x:c r="J16" s="40"/>
-      <x:c r="K16" s="35"/>
-      <x:c r="L16" s="35"/>
-      <x:c r="M16" s="35"/>
-      <x:c r="N16" s="35"/>
-      <x:c r="O16" s="35"/>
-      <x:c r="P16" s="35"/>
-      <x:c r="Q16" s="35"/>
-      <x:c r="R16" s="35"/>
-      <x:c r="S16" s="35"/>
-      <x:c r="T16" s="35"/>
-      <x:c r="U16" s="35"/>
-      <x:c r="V16" s="35"/>
-      <x:c r="W16" s="35"/>
-      <x:c r="X16" s="35"/>
-      <x:c r="Y16" s="35"/>
-      <x:c r="Z16" s="35"/>
-      <x:c r="AA16" s="35"/>
-      <x:c r="AB16" s="35"/>
-      <x:c r="AC16" s="35"/>
-      <x:c r="AD16" s="35"/>
-      <x:c r="AE16" s="35"/>
-      <x:c r="AF16" s="35"/>
-      <x:c r="AG16" s="35"/>
-      <x:c r="AH16" s="35"/>
-      <x:c r="AI16" s="35"/>
-      <x:c r="AJ16" s="35"/>
-      <x:c r="AK16" s="35"/>
-      <x:c r="AL16" s="35"/>
+      <x:c r="C16" s="48"/>
+      <x:c r="D16" s="48"/>
+      <x:c r="E16" s="48"/>
+      <x:c r="F16" s="48"/>
+      <x:c r="G16" s="48"/>
+      <x:c r="H16" s="48"/>
+      <x:c r="I16" s="48"/>
+      <x:c r="J16" s="48"/>
+      <x:c r="K16" s="48"/>
+      <x:c r="L16" s="48"/>
+      <x:c r="M16" s="48"/>
+      <x:c r="N16" s="48"/>
+      <x:c r="O16" s="48"/>
+      <x:c r="P16" s="48"/>
+      <x:c r="Q16" s="48"/>
+      <x:c r="R16" s="48"/>
+      <x:c r="S16" s="48"/>
+      <x:c r="T16" s="48"/>
+      <x:c r="U16" s="48"/>
+      <x:c r="V16" s="48"/>
+      <x:c r="W16" s="48"/>
+      <x:c r="X16" s="48"/>
+      <x:c r="Y16" s="48"/>
+      <x:c r="Z16" s="48"/>
+      <x:c r="AA16" s="48"/>
+      <x:c r="AB16" s="48"/>
+      <x:c r="AC16" s="48"/>
+      <x:c r="AD16" s="48"/>
+      <x:c r="AE16" s="48"/>
+      <x:c r="AF16" s="48"/>
+      <x:c r="AG16" s="48"/>
+      <x:c r="AH16" s="48"/>
+      <x:c r="AI16" s="48"/>
+      <x:c r="AJ16" s="48"/>
+      <x:c r="AK16" s="48"/>
+      <x:c r="AL16" s="48"/>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="46" t="str">
@@ -2775,42 +2886,42 @@
       <x:c r="B17" s="47" t="str">
         <x:v>Revisar documentação e consistência entre diagramas</x:v>
       </x:c>
-      <x:c r="C17" s="35"/>
-      <x:c r="D17" s="35"/>
-      <x:c r="E17" s="35"/>
-      <x:c r="F17" s="35"/>
-      <x:c r="G17" s="35"/>
-      <x:c r="H17" s="35"/>
-      <x:c r="I17" s="35"/>
-      <x:c r="J17" s="40"/>
-      <x:c r="K17" s="40"/>
-      <x:c r="L17" s="35"/>
-      <x:c r="M17" s="35"/>
-      <x:c r="N17" s="35"/>
-      <x:c r="O17" s="35"/>
-      <x:c r="P17" s="35"/>
-      <x:c r="Q17" s="35"/>
-      <x:c r="R17" s="35"/>
-      <x:c r="S17" s="35"/>
-      <x:c r="T17" s="35"/>
-      <x:c r="U17" s="35"/>
-      <x:c r="V17" s="35"/>
-      <x:c r="W17" s="35"/>
-      <x:c r="X17" s="35"/>
-      <x:c r="Y17" s="35"/>
-      <x:c r="Z17" s="35"/>
-      <x:c r="AA17" s="35"/>
-      <x:c r="AB17" s="35"/>
-      <x:c r="AC17" s="35"/>
-      <x:c r="AD17" s="35"/>
-      <x:c r="AE17" s="35"/>
-      <x:c r="AF17" s="35"/>
-      <x:c r="AG17" s="35"/>
-      <x:c r="AH17" s="35"/>
-      <x:c r="AI17" s="35"/>
-      <x:c r="AJ17" s="35"/>
-      <x:c r="AK17" s="35"/>
-      <x:c r="AL17" s="35"/>
+      <x:c r="C17" s="48"/>
+      <x:c r="D17" s="48"/>
+      <x:c r="E17" s="48"/>
+      <x:c r="F17" s="48"/>
+      <x:c r="G17" s="48"/>
+      <x:c r="H17" s="48"/>
+      <x:c r="I17" s="48"/>
+      <x:c r="J17" s="48"/>
+      <x:c r="K17" s="48"/>
+      <x:c r="L17" s="48"/>
+      <x:c r="M17" s="48"/>
+      <x:c r="N17" s="48"/>
+      <x:c r="O17" s="48"/>
+      <x:c r="P17" s="48"/>
+      <x:c r="Q17" s="48"/>
+      <x:c r="R17" s="48"/>
+      <x:c r="S17" s="48"/>
+      <x:c r="T17" s="48"/>
+      <x:c r="U17" s="48"/>
+      <x:c r="V17" s="48"/>
+      <x:c r="W17" s="48"/>
+      <x:c r="X17" s="48"/>
+      <x:c r="Y17" s="48"/>
+      <x:c r="Z17" s="48"/>
+      <x:c r="AA17" s="48"/>
+      <x:c r="AB17" s="48"/>
+      <x:c r="AC17" s="48"/>
+      <x:c r="AD17" s="48"/>
+      <x:c r="AE17" s="48"/>
+      <x:c r="AF17" s="48"/>
+      <x:c r="AG17" s="48"/>
+      <x:c r="AH17" s="48"/>
+      <x:c r="AI17" s="48"/>
+      <x:c r="AJ17" s="48"/>
+      <x:c r="AK17" s="48"/>
+      <x:c r="AL17" s="48"/>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
       <x:c r="A18" s="46" t="str">
@@ -2819,42 +2930,42 @@
       <x:c r="B18" s="47" t="str">
         <x:v>Preparar apresentação, metodologia e pré-banca</x:v>
       </x:c>
-      <x:c r="C18" s="35"/>
-      <x:c r="D18" s="35"/>
-      <x:c r="E18" s="35"/>
-      <x:c r="F18" s="35"/>
-      <x:c r="G18" s="35"/>
-      <x:c r="H18" s="35"/>
-      <x:c r="I18" s="35"/>
-      <x:c r="J18" s="40"/>
-      <x:c r="K18" s="40"/>
-      <x:c r="L18" s="35"/>
-      <x:c r="M18" s="35"/>
-      <x:c r="N18" s="35"/>
-      <x:c r="O18" s="35"/>
-      <x:c r="P18" s="35"/>
-      <x:c r="Q18" s="35"/>
-      <x:c r="R18" s="35"/>
-      <x:c r="S18" s="35"/>
-      <x:c r="T18" s="35"/>
-      <x:c r="U18" s="35"/>
-      <x:c r="V18" s="35"/>
-      <x:c r="W18" s="35"/>
-      <x:c r="X18" s="35"/>
-      <x:c r="Y18" s="35"/>
-      <x:c r="Z18" s="35"/>
-      <x:c r="AA18" s="35"/>
-      <x:c r="AB18" s="35"/>
-      <x:c r="AC18" s="35"/>
-      <x:c r="AD18" s="35"/>
-      <x:c r="AE18" s="35"/>
-      <x:c r="AF18" s="35"/>
-      <x:c r="AG18" s="35"/>
-      <x:c r="AH18" s="35"/>
-      <x:c r="AI18" s="35"/>
-      <x:c r="AJ18" s="35"/>
-      <x:c r="AK18" s="35"/>
-      <x:c r="AL18" s="35"/>
+      <x:c r="C18" s="48"/>
+      <x:c r="D18" s="48"/>
+      <x:c r="E18" s="48"/>
+      <x:c r="F18" s="48"/>
+      <x:c r="G18" s="48"/>
+      <x:c r="H18" s="48"/>
+      <x:c r="I18" s="48"/>
+      <x:c r="J18" s="48"/>
+      <x:c r="K18" s="48"/>
+      <x:c r="L18" s="48"/>
+      <x:c r="M18" s="48"/>
+      <x:c r="N18" s="48"/>
+      <x:c r="O18" s="48"/>
+      <x:c r="P18" s="48"/>
+      <x:c r="Q18" s="48"/>
+      <x:c r="R18" s="48"/>
+      <x:c r="S18" s="48"/>
+      <x:c r="T18" s="48"/>
+      <x:c r="U18" s="48"/>
+      <x:c r="V18" s="48"/>
+      <x:c r="W18" s="48"/>
+      <x:c r="X18" s="48"/>
+      <x:c r="Y18" s="48"/>
+      <x:c r="Z18" s="48"/>
+      <x:c r="AA18" s="48"/>
+      <x:c r="AB18" s="48"/>
+      <x:c r="AC18" s="48"/>
+      <x:c r="AD18" s="48"/>
+      <x:c r="AE18" s="48"/>
+      <x:c r="AF18" s="48"/>
+      <x:c r="AG18" s="48"/>
+      <x:c r="AH18" s="48"/>
+      <x:c r="AI18" s="48"/>
+      <x:c r="AJ18" s="48"/>
+      <x:c r="AK18" s="48"/>
+      <x:c r="AL18" s="48"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="31" t="inlineStr">
@@ -3436,6 +3547,81 @@
   <x:mergeCells>
     <x:mergeCell ref="A1:AL1"/>
   </x:mergeCells>
+  <x:conditionalFormatting sqref="C4:AL4">
+    <x:cfRule type="expression" dxfId="6" priority="1">
+      <x:formula>AND(C$3&lt;=Cronograma!$D9,C$3+6&gt;=Cronograma!$C9)</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="C5:AL5">
+    <x:cfRule type="expression" dxfId="7" priority="2">
+      <x:formula>AND(C$3&lt;=Cronograma!$D10,C$3+6&gt;=Cronograma!$C10)</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="C6:AL6">
+    <x:cfRule type="expression" dxfId="8" priority="3">
+      <x:formula>AND(C$3&lt;=Cronograma!$D11,C$3+6&gt;=Cronograma!$C11)</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="C7:AL7">
+    <x:cfRule type="expression" dxfId="9" priority="4">
+      <x:formula>AND(C$3&lt;=Cronograma!$D12,C$3+6&gt;=Cronograma!$C12)</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="C8:AL8">
+    <x:cfRule type="expression" dxfId="10" priority="5">
+      <x:formula>AND(C$3&lt;=Cronograma!$D13,C$3+6&gt;=Cronograma!$C13)</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="C9:AL9">
+    <x:cfRule type="expression" dxfId="11" priority="6">
+      <x:formula>AND(C$3&lt;=Cronograma!$D14,C$3+6&gt;=Cronograma!$C14)</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="C10:AL10">
+    <x:cfRule type="expression" dxfId="12" priority="7">
+      <x:formula>AND(C$3&lt;=Cronograma!$D15,C$3+6&gt;=Cronograma!$C15)</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="C11:AL11">
+    <x:cfRule type="expression" dxfId="13" priority="8">
+      <x:formula>AND(C$3&lt;=Cronograma!$D16,C$3+6&gt;=Cronograma!$C16)</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="C12:AL12">
+    <x:cfRule type="expression" dxfId="14" priority="9">
+      <x:formula>AND(C$3&lt;=Cronograma!$D17,C$3+6&gt;=Cronograma!$C17)</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="C13:AL13">
+    <x:cfRule type="expression" dxfId="15" priority="10">
+      <x:formula>AND(C$3&lt;=Cronograma!$D18,C$3+6&gt;=Cronograma!$C18)</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="C14:AL14">
+    <x:cfRule type="expression" dxfId="16" priority="11">
+      <x:formula>AND(C$3&lt;=Cronograma!$D19,C$3+6&gt;=Cronograma!$C19)</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="C15:AL15">
+    <x:cfRule type="expression" dxfId="17" priority="12">
+      <x:formula>AND(C$3&lt;=Cronograma!$D20,C$3+6&gt;=Cronograma!$C20)</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="C16:AL16">
+    <x:cfRule type="expression" dxfId="18" priority="13">
+      <x:formula>AND(C$3&lt;=Cronograma!$D21,C$3+6&gt;=Cronograma!$C21)</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="C17:AL17">
+    <x:cfRule type="expression" dxfId="19" priority="14">
+      <x:formula>AND(C$3&lt;=Cronograma!$D22,C$3+6&gt;=Cronograma!$C22)</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="C18:AL18">
+    <x:cfRule type="expression" dxfId="20" priority="15">
+      <x:formula>AND(C$3&lt;=Cronograma!$D23,C$3+6&gt;=Cronograma!$C23)</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: registra entregas concluidas no cronograma
</commit_message>
<xml_diff>
--- a/docs/planejamento/Cronograma_TCC_Gestao_Integrada.xlsx
+++ b/docs/planejamento/Cronograma_TCC_Gestao_Integrada.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cronograma" sheetId="1" r:id="R295fddf1f38e4229"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legenda" sheetId="2" r:id="R94cec3b7cde94ca7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gantt Semanal" sheetId="3" r:id="R5f3daae2dbf045c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cronograma" sheetId="1" r:id="R6d1bf37c2e4845c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legenda" sheetId="2" r:id="R15e00db56f7549f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gantt Semanal" sheetId="3" r:id="Re5a3d6265f32421b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -302,105 +302,105 @@
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9EAF7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9EAF7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9EAF7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9EAF7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9EAF7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -928,14 +928,14 @@
         <x:v>TCC1</x:v>
       </x:c>
       <x:c r="G9" s="6" t="str">
-        <x:v>Não iniciado</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
       <x:c r="H9" s="6"/>
       <x:c r="I9" s="6" t="str">
-        <x:v>Uma OP gerada automaticamente no registro de cada pedido</x:v>
+        <x:v>Fluxo macro: imagem, editável e documentação na main</x:v>
       </x:c>
       <x:c r="J9" s="8" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -962,10 +962,8 @@
           <x:t xml:space="preserve">TCC1</x:t>
         </x:is>
       </x:c>
-      <x:c r="G10" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Não iniciado</x:t>
-        </x:is>
+      <x:c r="G10" s="6" t="str">
+        <x:v>Concluído</x:v>
       </x:c>
       <x:c r="H10" s="6" t="inlineStr">
         <x:is>
@@ -973,10 +971,10 @@
         </x:is>
       </x:c>
       <x:c r="I10" s="6" t="str">
-        <x:v>Revisão baseada no macrofluxo</x:v>
+        <x:v>Escopo, requisitos e regras na main</x:v>
       </x:c>
       <x:c r="J10" s="8" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
@@ -1003,10 +1001,8 @@
           <x:t xml:space="preserve">TCC1</x:t>
         </x:is>
       </x:c>
-      <x:c r="G11" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Não iniciado</x:t>
-        </x:is>
+      <x:c r="G11" s="6" t="str">
+        <x:v>Concluído</x:v>
       </x:c>
       <x:c r="H11" s="6" t="inlineStr">
         <x:is>
@@ -1014,10 +1010,10 @@
         </x:is>
       </x:c>
       <x:c r="I11" s="6" t="str">
-        <x:v>Revisão coletiva da Issue #2</x:v>
+        <x:v>Catálogo de atores e casos de uso na main</x:v>
       </x:c>
       <x:c r="J11" s="8" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
@@ -1044,19 +1040,19 @@
           <x:t xml:space="preserve">TCC1</x:t>
         </x:is>
       </x:c>
-      <x:c r="G12" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Não iniciado</x:t>
-        </x:is>
+      <x:c r="G12" s="6" t="str">
+        <x:v>Concluído</x:v>
       </x:c>
       <x:c r="H12" s="6" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve"/>
         </x:is>
       </x:c>
-      <x:c r="I12" s="6"/>
+      <x:c r="I12" s="6" t="str">
+        <x:v>Diagrama, editável e descrições na main</x:v>
+      </x:c>
       <x:c r="J12" s="8" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
docs: corrige escala percentual do progresso
</commit_message>
<xml_diff>
--- a/docs/planejamento/Cronograma_TCC_Gestao_Integrada.xlsx
+++ b/docs/planejamento/Cronograma_TCC_Gestao_Integrada.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cronograma" sheetId="1" r:id="R6d1bf37c2e4845c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legenda" sheetId="2" r:id="R15e00db56f7549f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gantt Semanal" sheetId="3" r:id="Re5a3d6265f32421b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cronograma" sheetId="1" r:id="Rc2491c05ceba4382"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legenda" sheetId="2" r:id="Re401b293a05c42ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gantt Semanal" sheetId="3" r:id="R87af1e4313ad41ac"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -935,7 +935,7 @@
         <x:v>Fluxo macro: imagem, editável e documentação na main</x:v>
       </x:c>
       <x:c r="J9" s="8" t="n">
-        <x:v>100</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -974,7 +974,7 @@
         <x:v>Escopo, requisitos e regras na main</x:v>
       </x:c>
       <x:c r="J10" s="8" t="n">
-        <x:v>100</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
@@ -1013,7 +1013,7 @@
         <x:v>Catálogo de atores e casos de uso na main</x:v>
       </x:c>
       <x:c r="J11" s="8" t="n">
-        <x:v>100</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
@@ -1052,7 +1052,7 @@
         <x:v>Diagrama, editável e descrições na main</x:v>
       </x:c>
       <x:c r="J12" s="8" t="n">
-        <x:v>100</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">

</xml_diff>